<commit_message>
update progress excel in doc folder.
</commit_message>
<xml_diff>
--- a/Doc/進度.xlsx
+++ b/Doc/進度.xlsx
@@ -283,10 +283,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>進行中</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>將語音控制改為中文輸入</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -300,6 +296,10 @@
   </si>
   <si>
     <t>初步宣告vendor-defined成功並可回傳資料並在LCD上顯示文字</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>完成</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -878,7 +878,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -951,7 +951,7 @@
         <v>46247</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E2" s="15"/>
       <c r="F2" s="7" t="s">
@@ -975,7 +975,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="33">
+    <row r="3" spans="1:13">
       <c r="A3" s="4"/>
       <c r="B3" s="19"/>
       <c r="C3" s="20"/>
@@ -1050,10 +1050,10 @@
         <v>46314</v>
       </c>
       <c r="L5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="M5" s="9" t="s">
         <v>29</v>
-      </c>
-      <c r="M5" s="9" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1084,7 +1084,7 @@
       <c r="D7" s="6"/>
       <c r="E7" s="16"/>
       <c r="F7" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>12</v>
@@ -1107,7 +1107,7 @@
       <c r="D8" s="5"/>
       <c r="E8" s="18"/>
       <c r="F8" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>17</v>

</xml_diff>